<commit_message>
Alhamdulillah Nice work done for user and user password.
</commit_message>
<xml_diff>
--- a/RxForEyeIPD/Files/01. WithoutPrimaryAndForeignKey/TableCreateWithoutPrimaryAndForeignKey.xlsx
+++ b/RxForEyeIPD/Files/01. WithoutPrimaryAndForeignKey/TableCreateWithoutPrimaryAndForeignKey.xlsx
@@ -1444,13 +1444,13 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1921,34 +1921,34 @@
       <c r="B15" s="21"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B16" s="22"/>
+      <c r="B16" s="20"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="20" t="s">
         <v>105</v>
       </c>
-      <c r="B17" s="22"/>
+      <c r="B17" s="20"/>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="20" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="22"/>
+      <c r="B18" s="20"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="B19" s="22"/>
+      <c r="B19" s="20"/>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="B20" s="22"/>
+      <c r="B20" s="20"/>
     </row>
     <row r="21" spans="1:3" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A21" s="21" t="s">
@@ -1957,22 +1957,22 @@
       <c r="B21" s="21"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="B22" s="22"/>
+      <c r="B22" s="20"/>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="20" t="s">
         <v>111</v>
       </c>
-      <c r="B23" s="22"/>
+      <c r="B23" s="20"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="20" t="s">
         <v>112</v>
       </c>
-      <c r="B24" s="22"/>
+      <c r="B24" s="20"/>
     </row>
     <row r="28" spans="1:3" ht="17.25" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
@@ -1980,10 +1980,10 @@
       </c>
     </row>
     <row r="29" spans="1:3" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="20" t="s">
+      <c r="A29" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="20"/>
+      <c r="B29" s="22"/>
     </row>
     <row r="30" spans="1:3" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
@@ -2138,17 +2138,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A20:B20"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A18:B18"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>